<commit_message>
-- VF metadata structure added
</commit_message>
<xml_diff>
--- a/examples/sandbox/KG_standard/input/Standard_KG_template.xlsx
+++ b/examples/sandbox/KG_standard/input/Standard_KG_template.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uantwerpen-my.sharepoint.com/personal/bvanacker_ad_ua_ac_be/Documents/Documenten/00_UA/02_Projects/03_SAIfety/99_RemoteRepositories/vfWorks/examples/sandbox/KG_standard/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="250" documentId="11_AD4DB114E441178AC67DF4240E14F5EC693EDF12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1B634F1-B887-4D21-8FBB-62A9511FFCEA}"/>
+  <xr:revisionPtr revIDLastSave="252" documentId="11_AD4DB114E441178AC67DF4240E14F5EC693EDF12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EED72D7-81AF-472B-B87E-51841F76AB8D}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5460" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="trace" sheetId="1" r:id="rId1"/>
+    <sheet name="TRACE" sheetId="1" r:id="rId1"/>
     <sheet name="OBS" sheetId="5" r:id="rId2"/>
     <sheet name="LBS" sheetId="2" r:id="rId3"/>
     <sheet name="WBS" sheetId="3" r:id="rId4"/>
     <sheet name="WP" sheetId="7" r:id="rId5"/>
-    <sheet name="metrics" sheetId="4" r:id="rId6"/>
+    <sheet name="METRIC" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -388,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -458,9 +458,6 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -746,15 +743,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" customWidth="1"/>
-    <col min="4" max="4" width="40.42578125" customWidth="1"/>
+    <col min="3" max="3" width="42.88671875" customWidth="1"/>
+    <col min="4" max="4" width="40.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -776,15 +773,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DFE62D2-911D-4EED-96FE-5E969A4040A6}">
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.140625" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -798,151 +795,151 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="9"/>
       <c r="D2" s="7"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="9"/>
       <c r="D3" s="7"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="7"/>
       <c r="B4" s="8"/>
       <c r="C4" s="9"/>
       <c r="D4" s="7"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
       <c r="B5" s="8"/>
       <c r="C5" s="9"/>
       <c r="D5" s="7"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="7"/>
       <c r="B6" s="8"/>
       <c r="C6" s="9"/>
       <c r="D6" s="7"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
       <c r="B7" s="8"/>
       <c r="C7" s="9"/>
       <c r="D7" s="7"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="7"/>
       <c r="B8" s="8"/>
       <c r="C8" s="9"/>
       <c r="D8" s="7"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="7"/>
       <c r="B9" s="8"/>
       <c r="C9" s="9"/>
       <c r="D9" s="7"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
       <c r="B10" s="8"/>
       <c r="C10" s="9"/>
       <c r="D10" s="7"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
       <c r="B11" s="8"/>
       <c r="C11" s="9"/>
       <c r="D11" s="7"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="7"/>
       <c r="B12" s="8"/>
       <c r="C12" s="9"/>
       <c r="D12" s="7"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
       <c r="D13" s="7"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="9"/>
       <c r="D14" s="7"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
       <c r="D15" s="7"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>
       <c r="D16" s="7"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="9"/>
       <c r="D17" s="7"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="9"/>
       <c r="D18" s="7"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
       <c r="D19" s="7"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="7"/>
       <c r="B20" s="8"/>
       <c r="C20" s="9"/>
       <c r="D20" s="7"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="7"/>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
       <c r="D21" s="7"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
       <c r="B22" s="8"/>
       <c r="C22" s="9"/>
       <c r="D22" s="7"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="7"/>
       <c r="B23" s="8"/>
       <c r="C23" s="9"/>
       <c r="D23" s="7"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="7"/>
       <c r="B24" s="8"/>
       <c r="C24" s="9"/>
       <c r="D24" s="7"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="7"/>
       <c r="B25" s="8"/>
       <c r="C25" s="9"/>
       <c r="D25" s="7"/>
     </row>
-    <row r="26" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="10"/>
       <c r="B26" s="11"/>
       <c r="C26" s="12"/>
@@ -956,14 +953,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{185DBFE0-8C88-4565-B6AF-294BB3782FCA}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="32.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="32.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -974,147 +971,147 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
     </row>
-    <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -1127,17 +1124,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BA91118-3A2D-4F2D-8540-B700E2E8AB4E}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" customWidth="1"/>
-    <col min="3" max="3" width="46.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="7" width="26.28515625" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.44140625" customWidth="1"/>
+    <col min="3" max="3" width="46.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" customWidth="1"/>
+    <col min="5" max="5" width="17.88671875" customWidth="1"/>
+    <col min="6" max="7" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>11</v>
       </c>
@@ -1160,7 +1157,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -1169,7 +1166,7 @@
       <c r="F2" s="8"/>
       <c r="G2" s="26"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -1178,7 +1175,7 @@
       <c r="F3" s="8"/>
       <c r="G3" s="26"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -1187,7 +1184,7 @@
       <c r="F4" s="8"/>
       <c r="G4" s="26"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -1196,7 +1193,7 @@
       <c r="F5" s="8"/>
       <c r="G5" s="26"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -1205,7 +1202,7 @@
       <c r="F6" s="8"/>
       <c r="G6" s="26"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -1214,7 +1211,7 @@
       <c r="F7" s="8"/>
       <c r="G7" s="26"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -1223,7 +1220,7 @@
       <c r="F8" s="8"/>
       <c r="G8" s="26"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -1232,7 +1229,7 @@
       <c r="F9" s="8"/>
       <c r="G9" s="26"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -1241,7 +1238,7 @@
       <c r="F10" s="8"/>
       <c r="G10" s="26"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -1250,7 +1247,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="26"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -1259,7 +1256,7 @@
       <c r="F12" s="8"/>
       <c r="G12" s="26"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -1268,7 +1265,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="26"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -1277,7 +1274,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="26"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -1286,7 +1283,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="26"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -1295,7 +1292,7 @@
       <c r="F16" s="8"/>
       <c r="G16" s="26"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1304,7 +1301,7 @@
       <c r="F17" s="8"/>
       <c r="G17" s="26"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -1313,7 +1310,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="26"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -1322,7 +1319,7 @@
       <c r="F19" s="8"/>
       <c r="G19" s="26"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1331,7 +1328,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="26"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1340,7 +1337,7 @@
       <c r="F21" s="8"/>
       <c r="G21" s="26"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1349,7 +1346,7 @@
       <c r="F22" s="8"/>
       <c r="G22" s="26"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -1358,7 +1355,7 @@
       <c r="F23" s="8"/>
       <c r="G23" s="26"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1367,7 +1364,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="26"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -1376,7 +1373,7 @@
       <c r="F25" s="8"/>
       <c r="G25" s="26"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -1385,7 +1382,7 @@
       <c r="F26" s="8"/>
       <c r="G26" s="26"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -1394,7 +1391,7 @@
       <c r="F27" s="8"/>
       <c r="G27" s="26"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -1403,7 +1400,7 @@
       <c r="F28" s="8"/>
       <c r="G28" s="26"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -1412,7 +1409,7 @@
       <c r="F29" s="8"/>
       <c r="G29" s="26"/>
     </row>
-    <row r="30" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -1429,16 +1426,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{764AB8CB-FFAE-476A-97FC-AE47A0587795}">
   <dimension ref="A1:H30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="26.28515625" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" customWidth="1"/>
+    <col min="1" max="3" width="26.33203125" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" customWidth="1"/>
+    <col min="5" max="5" width="23.109375" customWidth="1"/>
     <col min="6" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
         <v>17</v>
       </c>
@@ -1464,7 +1461,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="26"/>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -1474,7 +1471,7 @@
       <c r="G2" s="30"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="26"/>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -1484,7 +1481,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="26"/>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -1494,7 +1491,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="26"/>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
@@ -1504,7 +1501,7 @@
       <c r="G5" s="8"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="26"/>
       <c r="B6" s="26"/>
       <c r="C6" s="26"/>
@@ -1514,7 +1511,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="26"/>
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
@@ -1524,7 +1521,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="26"/>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -1534,7 +1531,7 @@
       <c r="G8" s="8"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="26"/>
       <c r="B9" s="26"/>
       <c r="C9" s="26"/>
@@ -1544,7 +1541,7 @@
       <c r="G9" s="8"/>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="26"/>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
@@ -1554,7 +1551,7 @@
       <c r="G10" s="8"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="26"/>
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
@@ -1564,7 +1561,7 @@
       <c r="G11" s="8"/>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="26"/>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
@@ -1574,7 +1571,7 @@
       <c r="G12" s="8"/>
       <c r="H12" s="7"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
@@ -1584,7 +1581,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="26"/>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
@@ -1594,7 +1591,7 @@
       <c r="G14" s="8"/>
       <c r="H14" s="7"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="26"/>
       <c r="B15" s="26"/>
       <c r="C15" s="26"/>
@@ -1604,7 +1601,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="7"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="26"/>
       <c r="B16" s="26"/>
       <c r="C16" s="26"/>
@@ -1614,7 +1611,7 @@
       <c r="G16" s="8"/>
       <c r="H16" s="7"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
@@ -1624,7 +1621,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="7"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -1634,7 +1631,7 @@
       <c r="G18" s="8"/>
       <c r="H18" s="7"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="26"/>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -1644,7 +1641,7 @@
       <c r="G19" s="8"/>
       <c r="H19" s="7"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="26"/>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
@@ -1654,7 +1651,7 @@
       <c r="G20" s="8"/>
       <c r="H20" s="7"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="26"/>
       <c r="B21" s="26"/>
       <c r="C21" s="26"/>
@@ -1664,7 +1661,7 @@
       <c r="G21" s="8"/>
       <c r="H21" s="7"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="26"/>
       <c r="B22" s="26"/>
       <c r="C22" s="26"/>
@@ -1674,7 +1671,7 @@
       <c r="G22" s="8"/>
       <c r="H22" s="7"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="26"/>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
@@ -1684,7 +1681,7 @@
       <c r="G23" s="8"/>
       <c r="H23" s="7"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="26"/>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
@@ -1694,7 +1691,7 @@
       <c r="G24" s="8"/>
       <c r="H24" s="7"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="26"/>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -1704,7 +1701,7 @@
       <c r="G25" s="8"/>
       <c r="H25" s="7"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="26"/>
       <c r="B26" s="26"/>
       <c r="C26" s="26"/>
@@ -1714,7 +1711,7 @@
       <c r="G26" s="8"/>
       <c r="H26" s="7"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="26"/>
       <c r="B27" s="26"/>
       <c r="C27" s="26"/>
@@ -1724,7 +1721,7 @@
       <c r="G27" s="8"/>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="26"/>
       <c r="B28" s="26"/>
       <c r="C28" s="26"/>
@@ -1734,7 +1731,7 @@
       <c r="G28" s="8"/>
       <c r="H28" s="7"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="26"/>
       <c r="B29" s="26"/>
       <c r="C29" s="26"/>
@@ -1744,7 +1741,7 @@
       <c r="G29" s="8"/>
       <c r="H29" s="7"/>
     </row>
-    <row r="30" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="27"/>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
@@ -1762,22 +1759,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB022A34-B06E-4EF5-A197-6853861BF3C6}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D1" s="1" t="s">

</xml_diff>